<commit_message>
-- fixing age_des_type additional space mistake
</commit_message>
<xml_diff>
--- a/background_files/age_des_types.xlsx
+++ b/background_files/age_des_types.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\Projects\הסעת המונים\01_שלב ה\קבצי עבודה\תחזיות_דמוגרפיות\תחזיות_2050\התפלגות גילים\backround_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\advas\Documents\create_forecast_ad_hoc\background_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{348A0438-1117-4E6D-8C91-FF93D02A0D6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11880"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="45">
   <si>
     <t>classification_name</t>
   </si>
@@ -102,15 +103,9 @@
     <t>מתנחלי בינוני</t>
   </si>
   <si>
-    <t xml:space="preserve">מתנחלי מאוזן </t>
-  </si>
-  <si>
     <t>מתנחלי מבוגר</t>
   </si>
   <si>
-    <t xml:space="preserve">מתנחלי צעיר </t>
-  </si>
-  <si>
     <t>ערבי בינוני</t>
   </si>
   <si>
@@ -154,12 +149,18 @@
   </si>
   <si>
     <t>age_cycle</t>
+  </si>
+  <si>
+    <t>מתנחלי מאוזן</t>
+  </si>
+  <si>
+    <t>מתנחלי צעיר</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -233,7 +234,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -302,33 +303,33 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="טבלה1" displayName="טבלה1" ref="A1:U16" totalsRowShown="0" headerRowDxfId="1">
-  <autoFilter ref="A1:U16"/>
-  <sortState ref="A2:U16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="טבלה1" displayName="טבלה1" ref="A1:U16" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A1:U16" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:U16">
     <sortCondition ref="A1:A16"/>
   </sortState>
   <tableColumns count="21">
-    <tableColumn id="1" name="classification_name"/>
-    <tableColumn id="2" name="pop_0" dataCellStyle="Percent"/>
-    <tableColumn id="11" name="pop_5" dataDxfId="0" dataCellStyle="Percent"/>
-    <tableColumn id="3" name="pop_10" dataCellStyle="Percent"/>
-    <tableColumn id="4" name="pop_15" dataCellStyle="Percent"/>
-    <tableColumn id="5" name="pop_20" dataCellStyle="Percent"/>
-    <tableColumn id="6" name="pop_25" dataCellStyle="Percent"/>
-    <tableColumn id="7" name="pop_30" dataCellStyle="Percent"/>
-    <tableColumn id="8" name="pop_35" dataCellStyle="Percent"/>
-    <tableColumn id="9" name="pop_40" dataCellStyle="Percent"/>
-    <tableColumn id="10" name="pop_45" dataCellStyle="Percent"/>
-    <tableColumn id="12" name="pop_50" dataCellStyle="Percent"/>
-    <tableColumn id="13" name="pop_55" dataCellStyle="Percent"/>
-    <tableColumn id="14" name="pop_60" dataCellStyle="Percent"/>
-    <tableColumn id="15" name="pop_65" dataCellStyle="Percent"/>
-    <tableColumn id="16" name="pop_70" dataCellStyle="Percent"/>
-    <tableColumn id="17" name="pop_75up" dataCellStyle="Percent"/>
-    <tableColumn id="18" name="hh_size"/>
-    <tableColumn id="19" name="sector"/>
-    <tableColumn id="20" name="type"/>
-    <tableColumn id="21" name="age_cycle"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="classification_name"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="pop_0" dataCellStyle="Percent"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="pop_5" dataDxfId="0" dataCellStyle="Percent"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="pop_10" dataCellStyle="Percent"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="pop_15" dataCellStyle="Percent"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="pop_20" dataCellStyle="Percent"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="pop_25" dataCellStyle="Percent"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="pop_30" dataCellStyle="Percent"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="pop_35" dataCellStyle="Percent"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="pop_40" dataCellStyle="Percent"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="pop_45" dataCellStyle="Percent"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="pop_50" dataCellStyle="Percent"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="pop_55" dataCellStyle="Percent"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="pop_60" dataCellStyle="Percent"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="pop_65" dataCellStyle="Percent"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="pop_70" dataCellStyle="Percent"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="pop_75up" dataCellStyle="Percent"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="hh_size"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="sector"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="type"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="age_cycle"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -618,7 +619,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U16"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -690,13 +691,13 @@
         <v>17</v>
       </c>
       <c r="S1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="T1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="T1" s="2" t="s">
-        <v>35</v>
-      </c>
       <c r="U1" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.2">
@@ -755,10 +756,10 @@
         <v>6.5</v>
       </c>
       <c r="S2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="T2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="U2">
         <v>2</v>
@@ -820,10 +821,10 @@
         <v>5.5</v>
       </c>
       <c r="S3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="T3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="U3">
         <v>3</v>
@@ -885,10 +886,10 @@
         <v>4.5</v>
       </c>
       <c r="S4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="T4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="U4">
         <v>4</v>
@@ -950,10 +951,10 @@
         <v>7</v>
       </c>
       <c r="S5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="T5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="U5">
         <v>1</v>
@@ -1015,10 +1016,10 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="S6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="T6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="U6">
         <v>4</v>
@@ -1080,10 +1081,10 @@
         <v>3.5</v>
       </c>
       <c r="S7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="T7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="U7">
         <v>3</v>
@@ -1145,10 +1146,10 @@
         <v>3.8</v>
       </c>
       <c r="S8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="T8" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="U8">
         <v>2</v>
@@ -1210,10 +1211,10 @@
         <v>4.2</v>
       </c>
       <c r="S9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="T9" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="U9">
         <v>1</v>
@@ -1275,10 +1276,10 @@
         <v>4.5</v>
       </c>
       <c r="S10" t="s">
+        <v>32</v>
+      </c>
+      <c r="T10" t="s">
         <v>34</v>
-      </c>
-      <c r="T10" t="s">
-        <v>36</v>
       </c>
       <c r="U10">
         <v>2</v>
@@ -1286,7 +1287,7 @@
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="B11" s="3">
         <v>0.10400881987286251</v>
@@ -1340,10 +1341,10 @@
         <v>4</v>
       </c>
       <c r="S11" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="T11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="U11">
         <v>3</v>
@@ -1351,7 +1352,7 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B12" s="3">
         <v>8.6889321954169735E-2</v>
@@ -1405,10 +1406,10 @@
         <v>3.5</v>
       </c>
       <c r="S12" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="T12" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="U12">
         <v>4</v>
@@ -1416,7 +1417,7 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="B13" s="3">
         <v>0.18052139695031971</v>
@@ -1470,10 +1471,10 @@
         <v>5</v>
       </c>
       <c r="S13" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="T13" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="U13">
         <v>1</v>
@@ -1481,7 +1482,7 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B14" s="3">
         <v>0.12312912903067159</v>
@@ -1535,10 +1536,10 @@
         <v>4</v>
       </c>
       <c r="S14" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="T14" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="U14">
         <v>2</v>
@@ -1546,7 +1547,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B15" s="3">
         <v>0.1099121071280659</v>
@@ -1600,10 +1601,10 @@
         <v>4.5</v>
       </c>
       <c r="S15" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="T15" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="U15">
         <v>3</v>
@@ -1611,7 +1612,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B16" s="3">
         <v>0.14032756747722899</v>
@@ -1665,10 +1666,10 @@
         <v>5.5</v>
       </c>
       <c r="S16" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="T16" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="U16">
         <v>1</v>

</xml_diff>